<commit_message>
Fix GitHub notebook styling and publish saved example results without FASTQs
</commit_message>
<xml_diff>
--- a/example/reference_results/1_data_integrity_check/data_integrity_check.xlsx
+++ b/example/reference_results/1_data_integrity_check/data_integrity_check.xlsx
@@ -549,130 +549,130 @@
     <t xml:space="preserve">Classification</t>
   </si>
   <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mock-Community_S280_L001_R1_001.fastq.gz</t>
+    <t xml:space="preserve">example/data/fastq/Mock-Community_S280_L001_R1_001.fastq.gz</t>
   </si>
   <si>
     <t xml:space="preserve">Forward</t>
   </si>
   <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mock-Community_S280_L001_R2_001.fastq.gz</t>
+    <t xml:space="preserve">example/data/fastq/Mock-Community_S280_L001_R2_001.fastq.gz</t>
   </si>
   <si>
     <t xml:space="preserve">Reverse</t>
   </si>
   <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-000_S188_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-000_S188_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-001_S189_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-001_S189_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-002_S190_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-002_S190_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-003_S191_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-003_S191_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-005_S193_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-005_S193_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-006_S194_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-006_S194_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-007_S195_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-007_S195_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-008_S196_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-008_S196_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-009_S197_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-009_S197_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-141_S207_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-141_S207_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-142_S208_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-142_S208_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-143_S209_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-143_S209_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-144_S210_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-144_S210_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-145_S211_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-145_S211_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-146_S212_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-146_S212_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-147_S213_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-147_S213_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-148_S214_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-148_S214_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-149_S215_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-149_S215_L001_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-150_S216_L001_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/fastq/Mouse-F3-Day-150_S216_L001_R2_001.fastq.gz</t>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-000_S188_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-000_S188_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-001_S189_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-001_S189_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-002_S190_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-002_S190_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-003_S191_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-003_S191_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-005_S193_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-005_S193_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-006_S194_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-006_S194_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-007_S195_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-007_S195_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-008_S196_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-008_S196_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-009_S197_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-009_S197_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-141_S207_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-141_S207_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-142_S208_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-142_S208_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-143_S209_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-143_S209_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-144_S210_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-144_S210_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-145_S211_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-145_S211_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-146_S212_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-146_S212_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-147_S213_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-147_S213_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-148_S214_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-148_S214_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-149_S215_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-149_S215_L001_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-150_S216_L001_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example/data/fastq/Mouse-F3-Day-150_S216_L001_R2_001.fastq.gz</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet</t>

</xml_diff>